<commit_message>
feat: update data processing and results handling for datacentra integration
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -1,27 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28720"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GithubClonefiles\datacentra_unitcommitment\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F268AB86-59B4-43C3-A9DB-9B499DD8FA4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
+    <workbookView xWindow="8736" yWindow="7140" windowWidth="34560" windowHeight="18600" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="units_frequencyparam"/>
-    <sheet r:id="rId2" sheetId="2" name="winds_frequencyparam"/>
-    <sheet r:id="rId3" sheetId="3" name="strogesystem_data"/>
-    <sheet r:id="rId4" sheetId="4" name="units_data"/>
-    <sheet r:id="rId5" sheetId="5" name="units_cost"/>
-    <sheet r:id="rId6" sheetId="6" name="branch_data"/>
-    <sheet r:id="rId7" sheetId="7" name="load_curve"/>
-    <sheet r:id="rId8" sheetId="8" name="load_data"/>
+    <sheet name="units_frequencyparam" sheetId="1" r:id="rId1"/>
+    <sheet name="winds_frequencyparam" sheetId="2" r:id="rId2"/>
+    <sheet name="strogesystem_data" sheetId="3" r:id="rId3"/>
+    <sheet name="units_data" sheetId="4" r:id="rId4"/>
+    <sheet name="units_cost" sheetId="5" r:id="rId5"/>
+    <sheet name="branch_data" sheetId="6" r:id="rId6"/>
+    <sheet name="load_curve" sheetId="7" r:id="rId7"/>
+    <sheet name="load_data" sheetId="8" r:id="rId8"/>
+    <sheet name="data_centra" sheetId="9" r:id="rId9"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="55">
   <si>
     <t>index</t>
   </si>
@@ -162,18 +169,49 @@
   </si>
   <si>
     <t>Rg(0.04,0.1)</t>
+  </si>
+  <si>
+    <t>p_max</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>p_min</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>locatebus</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>voltage_regulation</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>lambda</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>mu</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>idale</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>sv_constant</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -182,6 +220,20 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -192,7 +244,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -207,163 +259,186 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C4" displayName="表12" name="表12" id="1" totalsRowShown="0">
-  <autoFilter ref="A1:C4"/>
-  <tableColumns count="3">
-    <tableColumn name="index" id="1"/>
-    <tableColumn name="locate_bus" id="2"/>
-    <tableColumn name="percent" id="3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="表5" displayName="表5" ref="A1:G4" totalsRowShown="0">
+  <autoFilter ref="A1:G4" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="index"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Hg(3,9)"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Dg(0,0.02)"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Kg(0,1)"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Fg(0.15,0.4)"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Tg(6,14)"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Rg(0.04,0.1)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:B25" displayName="表11" name="表11" id="2" totalsRowShown="0">
-  <autoFilter ref="A1:B25"/>
-  <tableColumns count="2">
-    <tableColumn name="index" id="1"/>
-    <tableColumn name="p" id="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="表2" displayName="表2" ref="A1:F3" totalsRowShown="0">
+  <autoFilter ref="A1:F3" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Fcmodel"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Kw"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Rw"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Mw"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Dw"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Tw"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E8" displayName="表10" name="表10" id="3" totalsRowShown="0">
-  <autoFilter ref="A1:E8"/>
-  <tableColumns count="5">
-    <tableColumn name="index" id="1"/>
-    <tableColumn name="from" id="2"/>
-    <tableColumn name="to" id="3"/>
-    <tableColumn name="x" id="4"/>
-    <tableColumn name="p_max" id="5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="表3" displayName="表3" ref="A1:L2" totalsRowShown="0">
+  <autoFilter ref="A1:L2" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="index"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="locate_bus"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="q_max"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="q_min"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="pg_max"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="pd_min"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="p_0"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="charge_rate"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="discharge_rate"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="charge_effi"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="discharge_effi"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="lossing_effi"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H4" displayName="表7" name="表7" id="4" totalsRowShown="0">
-  <autoFilter ref="A1:H4"/>
-  <tableColumns count="8">
-    <tableColumn name="index" id="1"/>
-    <tableColumn name="Gens_c" id="2"/>
-    <tableColumn name="Gens_b" id="3"/>
-    <tableColumn name="Gens_a" id="4"/>
-    <tableColumn name="Gens_CD" id="5"/>
-    <tableColumn name="Gens_CU" id="6"/>
-    <tableColumn name="Gens_CU1" id="7"/>
-    <tableColumn name="Gens_Cold" id="8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="表6" displayName="表6" ref="A1:M4" totalsRowShown="0">
+  <autoFilter ref="A1:M4" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="index"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="locate_bus"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="p_max"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="p_min"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Gens_RD"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Gens_RU"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="Gens_SD"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Gens_SU"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Gens_TU"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="Gens_TD"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="Gens_x0"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="Gens_t0"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0300-00000D000000}" name="Gens_p0"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:M4" displayName="表6" name="表6" id="5" totalsRowShown="0">
-  <autoFilter ref="A1:M4"/>
-  <tableColumns count="13">
-    <tableColumn name="index" id="1"/>
-    <tableColumn name="locate_bus" id="2"/>
-    <tableColumn name="p_max" id="3"/>
-    <tableColumn name="p_min" id="4"/>
-    <tableColumn name="Gens_RD" id="5"/>
-    <tableColumn name="Gens_RU" id="6"/>
-    <tableColumn name="Gens_SD" id="7"/>
-    <tableColumn name="Gens_SU" id="8"/>
-    <tableColumn name="Gens_TU" id="9"/>
-    <tableColumn name="Gens_TD" id="10"/>
-    <tableColumn name="Gens_x0" id="11"/>
-    <tableColumn name="Gens_t0" id="12"/>
-    <tableColumn name="Gens_p0" id="13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="表7" displayName="表7" ref="A1:H4" totalsRowShown="0">
+  <autoFilter ref="A1:H4" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="index"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Gens_c"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Gens_b"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Gens_a"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Gens_CD"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="Gens_CU"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Gens_CU1"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="Gens_Cold"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:L2" displayName="表3" name="表3" id="6" totalsRowShown="0">
-  <autoFilter ref="A1:L2"/>
-  <tableColumns count="12">
-    <tableColumn name="index" id="1"/>
-    <tableColumn name="locate_bus" id="2"/>
-    <tableColumn name="q_max" id="3"/>
-    <tableColumn name="q_min" id="4"/>
-    <tableColumn name="pg_max" id="5"/>
-    <tableColumn name="pd_min" id="6"/>
-    <tableColumn name="p_0" id="7"/>
-    <tableColumn name="charge_rate" id="8"/>
-    <tableColumn name="discharge_rate" id="9"/>
-    <tableColumn name="charge_effi" id="10"/>
-    <tableColumn name="discharge_effi" id="11"/>
-    <tableColumn name="lossing_effi" id="12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="表10" displayName="表10" ref="A1:E8" totalsRowShown="0">
+  <autoFilter ref="A1:E8" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="index"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="from"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="to"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="x"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="p_max"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:F3" displayName="表2" name="表2" id="7" totalsRowShown="0">
-  <autoFilter ref="A1:F3"/>
-  <tableColumns count="6">
-    <tableColumn name="Fcmodel" id="1"/>
-    <tableColumn name="Kw" id="2"/>
-    <tableColumn name="Rw" id="3"/>
-    <tableColumn name="Mw" id="4"/>
-    <tableColumn name="Dw" id="5"/>
-    <tableColumn name="Tw" id="6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="表11" displayName="表11" ref="A1:B25" totalsRowShown="0">
+  <autoFilter ref="A1:B25" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="index"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="p"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:G4" displayName="表5" name="表5" id="8" totalsRowShown="0">
-  <autoFilter ref="A1:G4"/>
-  <tableColumns count="7">
-    <tableColumn name="index" id="1"/>
-    <tableColumn name="Hg(3,9)" id="2"/>
-    <tableColumn name="Dg(0,0.02)" id="3"/>
-    <tableColumn name="Kg(0,1)" id="4"/>
-    <tableColumn name="Fg(0.15,0.4)" id="5"/>
-    <tableColumn name="Tg(6,14)" id="6"/>
-    <tableColumn name="Rg(0.04,0.1)" id="7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="表12" displayName="表12" ref="A1:C4" totalsRowShown="0">
+  <autoFilter ref="A1:C4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="index"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="locate_bus"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="percent"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -372,10 +447,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -413,71 +488,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -505,7 +580,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -528,11 +603,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -541,13 +616,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -557,7 +632,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -566,7 +641,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -575,7 +650,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -583,10 +658,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -651,23 +726,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="8.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="8.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="4" width="11.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="3" width="9.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="12.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row r="1" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -690,7 +765,7 @@
         <v>46</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row r="2" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -698,7 +773,7 @@
         <v>7</v>
       </c>
       <c r="C2" s="2">
-        <v>0.061</v>
+        <v>6.0999999999999999E-2</v>
       </c>
       <c r="D2" s="2">
         <v>0.9</v>
@@ -713,7 +788,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+    <row r="3" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -736,7 +811,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+    <row r="4" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -744,7 +819,7 @@
         <v>3.5</v>
       </c>
       <c r="C4" s="2">
-        <v>0.181</v>
+        <v>0.18099999999999999</v>
       </c>
       <c r="D4" s="2">
         <v>0.98</v>
@@ -760,6 +835,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -768,22 +844,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="9.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="9.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="13.5546875" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
@@ -803,7 +876,7 @@
         <v>40</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -811,7 +884,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>0.07</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="D2" s="1">
         <v>0</v>
@@ -823,7 +896,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -837,13 +910,14 @@
         <v>3</v>
       </c>
       <c r="E3" s="2">
-        <v>0.067</v>
+        <v>6.7000000000000004E-2</v>
       </c>
       <c r="F3" s="2">
         <v>0.06</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -852,28 +926,25 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="3" width="8.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="3" width="10.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="3" width="9.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="3" width="6.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="4" width="11.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="3" width="13.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="4" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="3" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row r="1" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -911,7 +982,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row r="2" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -950,6 +1021,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -958,29 +1030,24 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:M4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="3" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="3" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="3" width="9.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="3" width="9.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="3" width="9.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="3" width="9.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="3" width="9.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="3" width="9.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="3" width="9.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="9.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="10" width="9.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.5546875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row r="1" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1021,7 +1088,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row r="2" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1062,7 +1129,7 @@
         <v>150</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+    <row r="3" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1103,7 +1170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+    <row r="4" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1145,6 +1212,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -1153,24 +1221,21 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="3" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="3" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="3" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="3" width="11.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="13.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="9.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1196,7 +1261,7 @@
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1207,7 +1272,7 @@
         <v>13.5</v>
       </c>
       <c r="D2" s="2">
-        <v>0.0004</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="E2" s="1">
         <v>560</v>
@@ -1222,7 +1287,7 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1233,7 +1298,7 @@
         <v>32.6</v>
       </c>
       <c r="D3" s="2">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="E3" s="1">
         <v>350</v>
@@ -1248,7 +1313,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>6</v>
       </c>
@@ -1256,10 +1321,10 @@
         <v>137.4</v>
       </c>
       <c r="C4" s="2">
-        <v>17.6</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="D4" s="2">
-        <v>0.005</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="E4" s="1">
         <v>260</v>
@@ -1275,6 +1340,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -1283,21 +1349,20 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="8.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="8.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1314,7 +1379,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1331,7 +1396,7 @@
         <v>200</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1342,13 +1407,13 @@
         <v>4</v>
       </c>
       <c r="D3" s="2">
-        <v>0.258</v>
+        <v>0.25800000000000001</v>
       </c>
       <c r="E3" s="1">
         <v>120</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1359,13 +1424,13 @@
         <v>4</v>
       </c>
       <c r="D4" s="2">
-        <v>0.197</v>
+        <v>0.19700000000000001</v>
       </c>
       <c r="E4" s="1">
         <v>120</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1376,13 +1441,13 @@
         <v>6</v>
       </c>
       <c r="D5" s="2">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="E5" s="1">
         <v>120</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row r="6" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1393,13 +1458,13 @@
         <v>6</v>
       </c>
       <c r="D6" s="2">
-        <v>0.018</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="E6" s="1">
         <v>120</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1410,13 +1475,13 @@
         <v>3</v>
       </c>
       <c r="D7" s="2">
-        <v>0.037</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="E7" s="1">
         <v>200</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1427,13 +1492,14 @@
         <v>5</v>
       </c>
       <c r="D8" s="2">
-        <v>0.037</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="E8" s="1">
         <v>120</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -1442,18 +1508,18 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1461,7 +1527,7 @@
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1469,7 +1535,7 @@
         <v>219.19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1477,7 +1543,7 @@
         <v>235.35</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1485,7 +1551,7 @@
         <v>234.67</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1493,7 +1559,7 @@
         <v>236.73</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1501,7 +1567,7 @@
         <v>239.06</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1509,7 +1575,7 @@
         <v>244.48</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1517,15 +1583,15 @@
         <v>273.39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="2">
-        <v>290.4</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+        <v>290.39999999999998</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1533,7 +1599,7 @@
         <v>283.56</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1541,7 +1607,7 @@
         <v>281.2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1549,7 +1615,7 @@
         <v>328.61</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1557,7 +1623,7 @@
         <v>328.1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1565,15 +1631,15 @@
         <v>326.18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
       <c r="B15" s="2">
-        <v>323.6</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+        <v>323.60000000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1581,15 +1647,15 @@
         <v>326.86</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
       <c r="B17" s="2">
-        <v>287.79</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+        <v>287.79000000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1597,7 +1663,7 @@
         <v>260</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -1605,7 +1671,7 @@
         <v>246.74</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1613,7 +1679,7 @@
         <v>255.97</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+    <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1621,7 +1687,7 @@
         <v>237.35</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+    <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -1629,7 +1695,7 @@
         <v>243.31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+    <row r="23" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -1637,7 +1703,7 @@
         <v>283.14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+    <row r="24" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -1645,7 +1711,7 @@
         <v>283.05</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+    <row r="25" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -1654,6 +1720,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -1662,19 +1729,19 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1685,7 +1752,7 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1696,7 +1763,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1707,7 +1774,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1719,9 +1786,288 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EE2AA48-EAC4-44C8-A371-1C9C338278CF}">
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.77734375" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>0.5</v>
+      </c>
+      <c r="D2">
+        <v>0.1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>0.05</v>
+      </c>
+      <c r="G2">
+        <v>0.3</v>
+      </c>
+      <c r="H2">
+        <v>0.5</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>0.5</v>
+      </c>
+      <c r="D3">
+        <v>0.1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>0.05</v>
+      </c>
+      <c r="G3">
+        <v>0.3</v>
+      </c>
+      <c r="H3">
+        <v>0.2</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>0.5</v>
+      </c>
+      <c r="D4">
+        <v>0.1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>0.05</v>
+      </c>
+      <c r="G4">
+        <v>0.3</v>
+      </c>
+      <c r="H4">
+        <v>0.1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>0.5</v>
+      </c>
+      <c r="D5">
+        <v>0.1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>0.05</v>
+      </c>
+      <c r="G5">
+        <v>0.3</v>
+      </c>
+      <c r="H5">
+        <v>0.3</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>0.5</v>
+      </c>
+      <c r="D6">
+        <v>0.1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>0.05</v>
+      </c>
+      <c r="G6">
+        <v>0.3</v>
+      </c>
+      <c r="H6">
+        <v>0.4</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>0.5</v>
+      </c>
+      <c r="D7">
+        <v>0.1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>0.05</v>
+      </c>
+      <c r="G7">
+        <v>0.3</v>
+      </c>
+      <c r="H7">
+        <v>0.4</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>0.5</v>
+      </c>
+      <c r="D8">
+        <v>0.1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>0.05</v>
+      </c>
+      <c r="G8">
+        <v>0.3</v>
+      </c>
+      <c r="H8">
+        <v>0.5</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>0.5</v>
+      </c>
+      <c r="D9">
+        <v>0.1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>0.05</v>
+      </c>
+      <c r="G9">
+        <v>0.3</v>
+      </c>
+      <c r="H9">
+        <v>0.2</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add stacked DCC λ plot PDF and log file for latexindent processing
- Generated a new PDF file: stacked_dcc_λ_plot.pdf, containing the stacked DCC λ plot.
- Created an indent log file: indent.log, detailing the processing steps and settings used by latexindent.pl.
- Noted a fatal error indicating the absence of the temporary LaTeX file during indentation.
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28720"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GithubClonefiles\datacentra_unitcommitment\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F268AB86-59B4-43C3-A9DB-9B499DD8FA4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9795628E-2995-41FD-B564-CBC60567BF62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8736" yWindow="7140" windowWidth="34560" windowHeight="18600" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6156" yWindow="2652" windowWidth="34560" windowHeight="18540" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="units_frequencyparam" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,20 @@
     <sheet name="load_data" sheetId="8" r:id="rId8"/>
     <sheet name="data_centra" sheetId="9" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -274,7 +287,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -292,9 +305,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -1821,10 +1831,10 @@
       <c r="E1" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>54</v>
       </c>
       <c r="H1" s="6" t="s">
@@ -1845,6 +1855,7 @@
         <v>0.5</v>
       </c>
       <c r="D2">
+        <f>C2*0.2</f>
         <v>0.1</v>
       </c>
       <c r="E2">
@@ -1868,13 +1879,14 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="D3">
-        <v>0.1</v>
+        <f t="shared" ref="D3:D9" si="0">C3*0.2</f>
+        <v>0.16000000000000003</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -1886,7 +1898,7 @@
         <v>0.3</v>
       </c>
       <c r="H3">
-        <v>0.2</v>
+        <v>0.75</v>
       </c>
       <c r="I3">
         <v>1</v>
@@ -1897,13 +1909,14 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C4">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="D4">
-        <v>0.1</v>
+        <f t="shared" si="0"/>
+        <v>8.0000000000000016E-2</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -1915,7 +1928,7 @@
         <v>0.3</v>
       </c>
       <c r="H4">
-        <v>0.1</v>
+        <v>0.8</v>
       </c>
       <c r="I4">
         <v>1</v>
@@ -1926,13 +1939,14 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="D5">
-        <v>0.1</v>
+        <f t="shared" si="0"/>
+        <v>0.12</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -1955,12 +1969,13 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C6">
         <v>0.5</v>
       </c>
       <c r="D6">
+        <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
       <c r="E6">
@@ -1984,13 +1999,14 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="D7">
-        <v>0.1</v>
+        <f t="shared" si="0"/>
+        <v>0.13999999999999999</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2013,13 +2029,14 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="D8">
-        <v>0.1</v>
+        <f t="shared" si="0"/>
+        <v>0.16000000000000003</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2031,7 +2048,7 @@
         <v>0.3</v>
       </c>
       <c r="H8">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="I8">
         <v>1</v>
@@ -2048,6 +2065,7 @@
         <v>0.5</v>
       </c>
       <c r="D9">
+        <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
       <c r="E9">

</xml_diff>

<commit_message>
Cleaned up nested git repo and staged all files
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29001"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GithubClonefiles\datacentra_unitcommitment\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9795628E-2995-41FD-B564-CBC60567BF62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D752D26-6C11-45D2-919D-555B330F6DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6156" yWindow="2652" windowWidth="34560" windowHeight="18540" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="46032" yWindow="-48" windowWidth="46176" windowHeight="25296" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="units_frequencyparam" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="load_curve" sheetId="7" r:id="rId7"/>
     <sheet name="load_data" sheetId="8" r:id="rId8"/>
     <sheet name="data_centra" sheetId="9" r:id="rId9"/>
+    <sheet name="data_centra_jobcurve" sheetId="11" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="63">
   <si>
     <t>index</t>
   </si>
@@ -214,13 +215,39 @@
   <si>
     <t>sv_constant</t>
     <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>ddc1</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>ddc3</t>
+  </si>
+  <si>
+    <t>ddc2</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>ddc4</t>
+  </si>
+  <si>
+    <t>ddc5</t>
+  </si>
+  <si>
+    <t>ddc6</t>
+  </si>
+  <si>
+    <t>ddc7</t>
+  </si>
+  <si>
+    <t>ddc8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -247,6 +274,12 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF098658"/>
+      <name val="Fira Code"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -287,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -307,11 +340,56 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF098658"/>
+        <name val="Fira Code"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -337,6 +415,23 @@
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Rg(0.04,0.1)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{0A59F1F9-2B5D-4F80-AC32-27B4A687FF14}" name="表9_11" displayName="表9_11" ref="A1:H25" totalsRowShown="0" headerRowDxfId="1" dataCellStyle="常规">
+  <autoFilter ref="A1:H25" xr:uid="{0A59F1F9-2B5D-4F80-AC32-27B4A687FF14}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{DC4C90B9-0622-43B9-87C2-5D6F7199A79B}" name="ddc1" dataCellStyle="常规"/>
+    <tableColumn id="2" xr3:uid="{CAAEA72F-ABD5-4884-AC59-E413F5A981FA}" name="ddc2" dataCellStyle="常规"/>
+    <tableColumn id="3" xr3:uid="{0A8CC222-BE97-4363-A95A-B42EB8CC1C4B}" name="ddc3" dataCellStyle="常规"/>
+    <tableColumn id="4" xr3:uid="{9B4840C3-DFB4-447B-ACE8-96FDA4CCD282}" name="ddc4" dataCellStyle="常规"/>
+    <tableColumn id="5" xr3:uid="{D94B6A20-061B-4D18-A822-D19485944BBF}" name="ddc5" dataCellStyle="常规"/>
+    <tableColumn id="6" xr3:uid="{DBC02789-5FEA-4EED-8009-E8D233DDF965}" name="ddc6" dataCellStyle="常规"/>
+    <tableColumn id="7" xr3:uid="{537286FB-53CC-482A-9160-89B8352CF77C}" name="ddc7" dataCellStyle="常规"/>
+    <tableColumn id="8" xr3:uid="{2F9EF304-B2F6-447B-AA3F-4631738F9ABC}" name="ddc8" dataCellStyle="常规"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -447,6 +542,24 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="index"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="locate_bus"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="percent"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{AEEF0582-A7F4-4ABA-8FB7-15B7BE3DE26A}" name="表9" displayName="表9" ref="A1:I9" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:I9" xr:uid="{AEEF0582-A7F4-4ABA-8FB7-15B7BE3DE26A}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{360A2F3B-8D6F-4517-8356-E387D15DC7DA}" name="index"/>
+    <tableColumn id="2" xr3:uid="{38F57155-323F-45F7-B0B7-DDD01F06ABF9}" name="locatebus"/>
+    <tableColumn id="3" xr3:uid="{19E7B5ED-C6D4-4DC2-8C96-E0D3960B5505}" name="p_max"/>
+    <tableColumn id="4" xr3:uid="{AE0308F2-8D58-48C9-BA1D-02F1CD65289E}" name="p_min"/>
+    <tableColumn id="5" xr3:uid="{016A6FA0-0051-40AB-9073-573F97E2C989}" name="voltage_regulation"/>
+    <tableColumn id="6" xr3:uid="{E30730FF-F9F6-46DD-851C-6BE776CA0183}" name="idale"/>
+    <tableColumn id="7" xr3:uid="{2CE4DEF4-D19C-4D8F-A9E7-945C209B421D}" name="sv_constant"/>
+    <tableColumn id="8" xr3:uid="{436AD4E2-1F8D-49BB-927D-2EBC96340E38}" name="lambda"/>
+    <tableColumn id="9" xr3:uid="{CF34ACC3-12EE-4BB3-B590-12108D4416E5}" name="mu"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -853,6 +966,671 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4A1C8E2-376F-40CE-8085-79B300A67654}">
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:8" ht="16.8" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="8">
+        <v>12</v>
+      </c>
+      <c r="B2" s="8">
+        <v>10</v>
+      </c>
+      <c r="C2" s="8">
+        <v>15</v>
+      </c>
+      <c r="D2" s="9">
+        <v>12.482132966521601</v>
+      </c>
+      <c r="E2" s="9">
+        <v>10.133014800908301</v>
+      </c>
+      <c r="F2" s="9">
+        <v>16.2559273794473</v>
+      </c>
+      <c r="G2" s="9">
+        <v>13.362420428952399</v>
+      </c>
+      <c r="H2" s="9">
+        <v>11.0834190775251</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>7</v>
+      </c>
+      <c r="B3" s="8">
+        <v>8</v>
+      </c>
+      <c r="C3" s="8">
+        <v>20</v>
+      </c>
+      <c r="D3" s="9">
+        <v>7.1846593308838003</v>
+      </c>
+      <c r="E3" s="9">
+        <v>8.46490005155745</v>
+      </c>
+      <c r="F3" s="9">
+        <v>20.134717571778001</v>
+      </c>
+      <c r="G3" s="9">
+        <v>8.66652267210711</v>
+      </c>
+      <c r="H3" s="9">
+        <v>9.1504913859912005</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>5</v>
+      </c>
+      <c r="B4" s="8">
+        <v>5</v>
+      </c>
+      <c r="C4" s="8">
+        <v>15</v>
+      </c>
+      <c r="D4" s="9">
+        <v>5.0492554517678299</v>
+      </c>
+      <c r="E4" s="9">
+        <v>5.2562607071320597</v>
+      </c>
+      <c r="F4" s="9">
+        <v>15.7989312195627</v>
+      </c>
+      <c r="G4" s="9">
+        <v>5.4918705375587296</v>
+      </c>
+      <c r="H4" s="9">
+        <v>6.5443466992042101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>0</v>
+      </c>
+      <c r="B5" s="8">
+        <v>0</v>
+      </c>
+      <c r="C5" s="8">
+        <v>10</v>
+      </c>
+      <c r="D5" s="9">
+        <v>0.76882121864844</v>
+      </c>
+      <c r="E5" s="9">
+        <v>0.21661069932951901</v>
+      </c>
+      <c r="F5" s="9">
+        <v>11.157421165438899</v>
+      </c>
+      <c r="G5" s="9">
+        <v>2.0762461708087399</v>
+      </c>
+      <c r="H5" s="9">
+        <v>1.1672273911711</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
+        <v>0</v>
+      </c>
+      <c r="B6" s="8">
+        <v>0</v>
+      </c>
+      <c r="C6" s="8">
+        <v>9</v>
+      </c>
+      <c r="D6" s="9">
+        <v>1.3661582168218001</v>
+      </c>
+      <c r="E6" s="9">
+        <v>1.4503987638129201</v>
+      </c>
+      <c r="F6" s="9">
+        <v>10.4202542162939</v>
+      </c>
+      <c r="G6" s="9">
+        <v>2.28809361523663</v>
+      </c>
+      <c r="H6" s="9">
+        <v>2.31060876860262</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>0</v>
+      </c>
+      <c r="B7" s="8">
+        <v>0</v>
+      </c>
+      <c r="C7" s="8">
+        <v>15</v>
+      </c>
+      <c r="D7" s="9">
+        <v>0.92195084482203404</v>
+      </c>
+      <c r="E7" s="9">
+        <v>0.84276609069757102</v>
+      </c>
+      <c r="F7" s="9">
+        <v>16.432142166946001</v>
+      </c>
+      <c r="G7" s="9">
+        <v>1.7706619832683901</v>
+      </c>
+      <c r="H7" s="9">
+        <v>0.86744253489736001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
+        <v>0</v>
+      </c>
+      <c r="B8" s="8">
+        <v>0</v>
+      </c>
+      <c r="C8" s="8">
+        <v>20</v>
+      </c>
+      <c r="D8" s="9">
+        <v>0.89627245036675696</v>
+      </c>
+      <c r="E8" s="9">
+        <v>0.80287811211428195</v>
+      </c>
+      <c r="F8" s="9">
+        <v>20.351015808577401</v>
+      </c>
+      <c r="G8" s="9">
+        <v>1.7243987776646399</v>
+      </c>
+      <c r="H8" s="9">
+        <v>1.0497722192183601</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>0</v>
+      </c>
+      <c r="B9" s="8">
+        <v>0</v>
+      </c>
+      <c r="C9" s="8">
+        <v>20</v>
+      </c>
+      <c r="D9" s="9">
+        <v>0.25938474383585503</v>
+      </c>
+      <c r="E9" s="9">
+        <v>1.46395204126779</v>
+      </c>
+      <c r="F9" s="9">
+        <v>20.8626202488628</v>
+      </c>
+      <c r="G9" s="9">
+        <v>1.26567514326965</v>
+      </c>
+      <c r="H9" s="9">
+        <v>2.4341948676989902</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
+        <v>3</v>
+      </c>
+      <c r="B10" s="8">
+        <v>0</v>
+      </c>
+      <c r="C10" s="8">
+        <v>20</v>
+      </c>
+      <c r="D10" s="9">
+        <v>4.3759517362571598</v>
+      </c>
+      <c r="E10" s="9">
+        <v>1.1834276278942999</v>
+      </c>
+      <c r="F10" s="9">
+        <v>20.794033617720402</v>
+      </c>
+      <c r="G10" s="9">
+        <v>4.4516506107180103</v>
+      </c>
+      <c r="H10" s="9">
+        <v>2.0343493603832501</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
+        <v>8</v>
+      </c>
+      <c r="B11" s="8">
+        <v>0</v>
+      </c>
+      <c r="C11" s="8">
+        <v>20</v>
+      </c>
+      <c r="D11" s="9">
+        <v>8.6733249985064909</v>
+      </c>
+      <c r="E11" s="9">
+        <v>0.48890549004623601</v>
+      </c>
+      <c r="F11" s="9">
+        <v>21.0307955492251</v>
+      </c>
+      <c r="G11" s="9">
+        <v>9.3742928556112304</v>
+      </c>
+      <c r="H11" s="9">
+        <v>1.1995187607139</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
+        <v>13</v>
+      </c>
+      <c r="B12" s="8">
+        <v>0</v>
+      </c>
+      <c r="C12" s="8">
+        <v>20</v>
+      </c>
+      <c r="D12" s="9">
+        <v>14.076146663390601</v>
+      </c>
+      <c r="E12" s="9">
+        <v>0.84394844120076296</v>
+      </c>
+      <c r="F12" s="9">
+        <v>20.560421462572101</v>
+      </c>
+      <c r="G12" s="9">
+        <v>15.536369893834101</v>
+      </c>
+      <c r="H12" s="9">
+        <v>2.2616215037593101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="8">
+        <v>15</v>
+      </c>
+      <c r="B13" s="8">
+        <v>0</v>
+      </c>
+      <c r="C13" s="8">
+        <v>20</v>
+      </c>
+      <c r="D13" s="9">
+        <v>15.3298218093441</v>
+      </c>
+      <c r="E13" s="9">
+        <v>0.62652086313991895</v>
+      </c>
+      <c r="F13" s="9">
+        <v>21.266670370993399</v>
+      </c>
+      <c r="G13" s="9">
+        <v>16.730851802151999</v>
+      </c>
+      <c r="H13" s="9">
+        <v>0.96564137427744001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="8">
+        <v>15</v>
+      </c>
+      <c r="B14" s="8">
+        <v>0</v>
+      </c>
+      <c r="C14" s="8">
+        <v>20</v>
+      </c>
+      <c r="D14" s="9">
+        <v>16.444577367495501</v>
+      </c>
+      <c r="E14" s="9">
+        <v>3.4083528755368603E-2</v>
+      </c>
+      <c r="F14" s="9">
+        <v>20.476619760813001</v>
+      </c>
+      <c r="G14" s="9">
+        <v>17.026390208689101</v>
+      </c>
+      <c r="H14" s="9">
+        <v>7.0652050809779002E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
+        <v>15</v>
+      </c>
+      <c r="B15" s="8">
+        <v>0</v>
+      </c>
+      <c r="C15" s="8">
+        <v>20</v>
+      </c>
+      <c r="D15" s="9">
+        <v>16.428349556905001</v>
+      </c>
+      <c r="E15" s="9">
+        <v>0.479613639881248</v>
+      </c>
+      <c r="F15" s="9">
+        <v>21.262630562738401</v>
+      </c>
+      <c r="G15" s="9">
+        <v>17.9136123261497</v>
+      </c>
+      <c r="H15" s="9">
+        <v>1.2444738852730599</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="8">
+        <v>13</v>
+      </c>
+      <c r="B16" s="8">
+        <v>0</v>
+      </c>
+      <c r="C16" s="8">
+        <v>20</v>
+      </c>
+      <c r="D16" s="9">
+        <v>13.8217300761054</v>
+      </c>
+      <c r="E16" s="9">
+        <v>1.26191783226417</v>
+      </c>
+      <c r="F16" s="9">
+        <v>21.1548958794776</v>
+      </c>
+      <c r="G16" s="9">
+        <v>14.6684784263136</v>
+      </c>
+      <c r="H16" s="9">
+        <v>1.5525566210136199</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="8">
+        <v>10</v>
+      </c>
+      <c r="B17" s="8">
+        <v>0</v>
+      </c>
+      <c r="C17" s="8">
+        <v>20</v>
+      </c>
+      <c r="D17" s="9">
+        <v>10.4414674345149</v>
+      </c>
+      <c r="E17" s="9">
+        <v>1.01949953180611</v>
+      </c>
+      <c r="F17" s="9">
+        <v>20.9071872518576</v>
+      </c>
+      <c r="G17" s="9">
+        <v>10.609924961660001</v>
+      </c>
+      <c r="H17" s="9">
+        <v>1.22629686438372</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="8">
+        <v>7</v>
+      </c>
+      <c r="B18" s="8">
+        <v>0</v>
+      </c>
+      <c r="C18" s="8">
+        <v>20</v>
+      </c>
+      <c r="D18" s="9">
+        <v>7.2880200171191802</v>
+      </c>
+      <c r="E18" s="9">
+        <v>8.5033964564166606E-2</v>
+      </c>
+      <c r="F18" s="9">
+        <v>20.069893422355499</v>
+      </c>
+      <c r="G18" s="9">
+        <v>7.4798379156685897</v>
+      </c>
+      <c r="H18" s="9">
+        <v>0.65676843148016195</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="8">
+        <v>10</v>
+      </c>
+      <c r="B19" s="8">
+        <v>0</v>
+      </c>
+      <c r="C19" s="8">
+        <v>20</v>
+      </c>
+      <c r="D19" s="9">
+        <v>11.2506358740174</v>
+      </c>
+      <c r="E19" s="9">
+        <v>1.2625780093475401</v>
+      </c>
+      <c r="F19" s="9">
+        <v>20.665234346450301</v>
+      </c>
+      <c r="G19" s="9">
+        <v>12.089448446815499</v>
+      </c>
+      <c r="H19" s="9">
+        <v>2.2101568643165002</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="8">
+        <v>13</v>
+      </c>
+      <c r="B20" s="8">
+        <v>0</v>
+      </c>
+      <c r="C20" s="8">
+        <v>20</v>
+      </c>
+      <c r="D20" s="9">
+        <v>14.2341769538761</v>
+      </c>
+      <c r="E20" s="9">
+        <v>0.615830519959228</v>
+      </c>
+      <c r="F20" s="9">
+        <v>20.0455982002645</v>
+      </c>
+      <c r="G20" s="9">
+        <v>15.7183461290381</v>
+      </c>
+      <c r="H20" s="9">
+        <v>1.7324962083717901</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="8">
+        <v>10</v>
+      </c>
+      <c r="B21" s="8">
+        <v>0</v>
+      </c>
+      <c r="C21" s="8">
+        <v>20</v>
+      </c>
+      <c r="D21" s="9">
+        <v>10.590835025496</v>
+      </c>
+      <c r="E21" s="9">
+        <v>0.21207605561232101</v>
+      </c>
+      <c r="F21" s="9">
+        <v>20.3387471836235</v>
+      </c>
+      <c r="G21" s="9">
+        <v>10.9457549312487</v>
+      </c>
+      <c r="H21" s="9">
+        <v>1.19563306082064</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="8">
+        <v>5</v>
+      </c>
+      <c r="B22" s="8">
+        <v>0</v>
+      </c>
+      <c r="C22" s="8">
+        <v>20</v>
+      </c>
+      <c r="D22" s="9">
+        <v>5.2748554128940901</v>
+      </c>
+      <c r="E22" s="9">
+        <v>1.0140788800426599</v>
+      </c>
+      <c r="F22" s="9">
+        <v>20.765366257793101</v>
+      </c>
+      <c r="G22" s="9">
+        <v>6.0302130280462398</v>
+      </c>
+      <c r="H22" s="9">
+        <v>1.4364740227828401</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="8">
+        <v>0</v>
+      </c>
+      <c r="B23" s="8">
+        <v>0</v>
+      </c>
+      <c r="C23" s="8">
+        <v>15</v>
+      </c>
+      <c r="D23" s="9">
+        <v>0.99956649592548696</v>
+      </c>
+      <c r="E23" s="9">
+        <v>1.9023323430054601E-2</v>
+      </c>
+      <c r="F23" s="9">
+        <v>16.189611542698199</v>
+      </c>
+      <c r="G23" s="9">
+        <v>1.627068398185</v>
+      </c>
+      <c r="H23" s="9">
+        <v>1.4476028239477601</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="8">
+        <v>0</v>
+      </c>
+      <c r="B24" s="8">
+        <v>0</v>
+      </c>
+      <c r="C24" s="8">
+        <v>5</v>
+      </c>
+      <c r="D24" s="9">
+        <v>1.12600404107181</v>
+      </c>
+      <c r="E24" s="9">
+        <v>0.85083274961590305</v>
+      </c>
+      <c r="F24" s="9">
+        <v>5.6067328740204703</v>
+      </c>
+      <c r="G24" s="9">
+        <v>1.65595510596778</v>
+      </c>
+      <c r="H24" s="9">
+        <v>1.6901554088944299</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="8">
+        <v>0</v>
+      </c>
+      <c r="B25" s="8">
+        <v>0</v>
+      </c>
+      <c r="C25" s="8">
+        <v>5</v>
+      </c>
+      <c r="D25" s="9">
+        <v>6.0273780028474701E-2</v>
+      </c>
+      <c r="E25" s="9">
+        <v>1.40849166565771</v>
+      </c>
+      <c r="F25" s="9">
+        <v>1.2156366665484799</v>
+      </c>
+      <c r="G25" s="9">
+        <v>0.70961608800254805</v>
+      </c>
+      <c r="H25" s="9">
+        <v>2.2085531331593899</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
@@ -1810,9 +2588,10 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.77734375" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
     <col min="5" max="5" width="19.33203125" customWidth="1"/>
     <col min="7" max="7" width="14.109375" customWidth="1"/>
+    <col min="8" max="8" width="9.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" x14ac:dyDescent="0.3">
@@ -1852,11 +2631,10 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>0.5</v>
+        <v>50</v>
       </c>
       <c r="D2">
-        <f>C2*0.2</f>
-        <v>0.1</v>
+        <v>10</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -1882,11 +2660,10 @@
         <v>2</v>
       </c>
       <c r="C3">
-        <v>0.8</v>
+        <v>30</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D9" si="0">C3*0.2</f>
-        <v>0.16000000000000003</v>
+        <v>6</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -1912,11 +2689,10 @@
         <v>6</v>
       </c>
       <c r="C4">
-        <v>0.4</v>
+        <v>80</v>
       </c>
       <c r="D4">
-        <f t="shared" si="0"/>
-        <v>8.0000000000000016E-2</v>
+        <v>16</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -1942,11 +2718,10 @@
         <v>2</v>
       </c>
       <c r="C5">
-        <v>0.6</v>
+        <v>60</v>
       </c>
       <c r="D5">
-        <f t="shared" si="0"/>
-        <v>0.12</v>
+        <v>12</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -1972,11 +2747,10 @@
         <v>6</v>
       </c>
       <c r="C6">
-        <v>0.5</v>
+        <v>60</v>
       </c>
       <c r="D6">
-        <f t="shared" si="0"/>
-        <v>0.1</v>
+        <v>12</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2002,11 +2776,10 @@
         <v>2</v>
       </c>
       <c r="C7">
-        <v>0.7</v>
+        <v>20</v>
       </c>
       <c r="D7">
-        <f t="shared" si="0"/>
-        <v>0.13999999999999999</v>
+        <v>4</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2032,11 +2805,10 @@
         <v>2</v>
       </c>
       <c r="C8">
-        <v>0.8</v>
+        <v>30</v>
       </c>
       <c r="D8">
-        <f t="shared" si="0"/>
-        <v>0.16000000000000003</v>
+        <v>6</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2062,11 +2834,10 @@
         <v>1</v>
       </c>
       <c r="C9">
-        <v>0.5</v>
+        <v>50</v>
       </c>
       <c r="D9">
-        <f t="shared" si="0"/>
-        <v>0.1</v>
+        <v>10</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2087,5 +2858,8 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>